<commit_message>
Update September report with August 2026 operations and warm-season analysis.
Refresh the WETA schedule from the latest operating record, add August SNOTEL plots and April–August climatology, and rewrite the report around a dry August at the La Sal targets.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/raw/WA25001_Flat_Iron_UT_HVG_Operating_Record_v01.xlsx
+++ b/data/raw/WA25001_Flat_Iron_UT_HVG_Operating_Record_v01.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="15">
   <si>
     <t>WA25001 Operating Times</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>Dry start</t>
+  </si>
+  <si>
+    <t>Shut down due to flood warnings</t>
   </si>
 </sst>
 </file>
@@ -2881,12 +2884,24 @@
       <c r="Z66" s="6"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="6"/>
-      <c r="B67" s="6"/>
-      <c r="C67" s="6"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="6"/>
-      <c r="F67" s="6"/>
+      <c r="A67" s="12">
+        <v>46264.0</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C67" s="9">
+        <v>1256.0</v>
+      </c>
+      <c r="D67" s="9">
+        <v>99.9</v>
+      </c>
+      <c r="E67" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="F67" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="G67" s="6"/>
       <c r="H67" s="6"/>
       <c r="I67" s="6"/>
@@ -2909,11 +2924,21 @@
       <c r="Z67" s="6"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="6"/>
-      <c r="B68" s="6"/>
-      <c r="C68" s="6"/>
-      <c r="D68" s="6"/>
-      <c r="E68" s="6"/>
+      <c r="A68" s="12">
+        <v>46267.0</v>
+      </c>
+      <c r="B68" s="9">
+        <v>1915.0</v>
+      </c>
+      <c r="C68" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E68" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F68" s="6"/>
       <c r="G68" s="6"/>
       <c r="H68" s="6"/>
@@ -2937,11 +2962,21 @@
       <c r="Z68" s="6"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="6"/>
-      <c r="B69" s="6"/>
-      <c r="C69" s="6"/>
-      <c r="D69" s="6"/>
-      <c r="E69" s="6"/>
+      <c r="A69" s="12">
+        <v>46268.0</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C69" s="9">
+        <v>1520.0</v>
+      </c>
+      <c r="D69" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E69" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F69" s="6"/>
       <c r="G69" s="6"/>
       <c r="H69" s="6"/>
@@ -2965,11 +3000,21 @@
       <c r="Z69" s="6"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="6"/>
-      <c r="B70" s="6"/>
-      <c r="C70" s="6"/>
-      <c r="D70" s="6"/>
-      <c r="E70" s="6"/>
+      <c r="A70" s="12">
+        <v>46276.0</v>
+      </c>
+      <c r="B70" s="9">
+        <v>2339.0</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E70" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F70" s="6"/>
       <c r="G70" s="6"/>
       <c r="H70" s="6"/>
@@ -2996,7 +3041,7 @@
       <c r="A71" s="6"/>
       <c r="B71" s="6"/>
       <c r="C71" s="6"/>
-      <c r="D71" s="6"/>
+      <c r="D71" s="9"/>
       <c r="E71" s="6"/>
       <c r="F71" s="6"/>
       <c r="G71" s="6"/>

</xml_diff>

<commit_message>
Update October report with September 2026 operations and precipitation.
Use the latest operating record, including flood-risk shutdowns, and count SNOTEL month totals from start-of-day accumulation so August includes September 1 and September stops before the water-year reset.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/raw/WA25001_Flat_Iron_UT_HVG_Operating_Record_v01.xlsx
+++ b/data/raw/WA25001_Flat_Iron_UT_HVG_Operating_Record_v01.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="17">
   <si>
     <t>WA25001 Operating Times</t>
   </si>
@@ -63,6 +63,12 @@
   </si>
   <si>
     <t>Shut down due to flood warnings</t>
+  </si>
+  <si>
+    <t>Shut down due to flood risk</t>
+  </si>
+  <si>
+    <t>Low humidity - Dry start</t>
   </si>
 </sst>
 </file>
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -152,6 +158,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="167" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -3038,12 +3047,24 @@
       <c r="Z70" s="6"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="6"/>
-      <c r="B71" s="6"/>
-      <c r="C71" s="6"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="6"/>
-      <c r="F71" s="6"/>
+      <c r="A71" s="12">
+        <v>46282.0</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C71" s="9">
+        <v>703.0</v>
+      </c>
+      <c r="D71" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E71" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="F71" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="G71" s="6"/>
       <c r="H71" s="6"/>
       <c r="I71" s="6"/>
@@ -3066,11 +3087,21 @@
       <c r="Z71" s="6"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="6"/>
-      <c r="B72" s="6"/>
-      <c r="C72" s="6"/>
-      <c r="D72" s="6"/>
-      <c r="E72" s="6"/>
+      <c r="A72" s="12">
+        <v>46286.0</v>
+      </c>
+      <c r="B72" s="9">
+        <v>1405.0</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="9">
+        <v>99.8</v>
+      </c>
+      <c r="E72" s="9">
+        <v>0.1</v>
+      </c>
       <c r="F72" s="6"/>
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
@@ -3094,12 +3125,24 @@
       <c r="Z72" s="6"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="6"/>
-      <c r="B73" s="6"/>
-      <c r="C73" s="6"/>
-      <c r="D73" s="6"/>
-      <c r="E73" s="6"/>
-      <c r="F73" s="6"/>
+      <c r="A73" s="12">
+        <v>46292.0</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C73" s="9">
+        <v>936.0</v>
+      </c>
+      <c r="D73" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E73" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="G73" s="6"/>
       <c r="H73" s="6"/>
       <c r="I73" s="6"/>
@@ -3122,12 +3165,24 @@
       <c r="Z73" s="6"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="6"/>
-      <c r="B74" s="6"/>
-      <c r="C74" s="6"/>
-      <c r="D74" s="6"/>
-      <c r="E74" s="6"/>
-      <c r="F74" s="6"/>
+      <c r="A74" s="12">
+        <v>46302.0</v>
+      </c>
+      <c r="B74" s="9">
+        <v>1347.0</v>
+      </c>
+      <c r="C74" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="9">
+        <v>99.8</v>
+      </c>
+      <c r="E74" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="F74" s="9" t="s">
+        <v>16</v>
+      </c>
       <c r="G74" s="6"/>
       <c r="H74" s="6"/>
       <c r="I74" s="6"/>
@@ -3150,12 +3205,24 @@
       <c r="Z74" s="6"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6"/>
-      <c r="C75" s="6"/>
-      <c r="D75" s="6"/>
-      <c r="E75" s="6"/>
-      <c r="F75" s="6"/>
+      <c r="A75" s="10">
+        <v>46308.0</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C75" s="9">
+        <v>908.0</v>
+      </c>
+      <c r="D75" s="9">
+        <v>99.7</v>
+      </c>
+      <c r="E75" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="F75" s="14" t="s">
+        <v>15</v>
+      </c>
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
       <c r="I75" s="6"/>

</xml_diff>